<commit_message>
Leads: 2026-10-05 00:08 UTC (cycle 196)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,66 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>24 HRS- Palmdale Sewer Repair</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>mrplumbingdraincleaning.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.mrplumbingdraincleaning.com/ca/palmdale/sewerrepair.php</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>But If</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>palmdale@mrplumbingdraincleaning.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>661-427-2602</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Palmdale CA</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>88</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>sewer repair Palmdale CA</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 00:09 UTC (cycle 197)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -623,6 +623,66 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Emergency Plumber Orlando | Choice Plumbing | (407) 422-7443</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>choiceplumbingorlando.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://choiceplumbingorlando.com/emergency</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Central Florida</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>nickshif@gmail.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(407) 422-7443</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Orlando FL</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>emergency plumber Orlando FL</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 00:14 UTC (cycle 200)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -683,6 +683,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>roofingpros7.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://roofingpros7.com/metal-roofing.php</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Call Now</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>roofingpros.inc.c@gmail.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(559) 730-8511</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Fresno CA</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Fresno CA</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 05:26 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -743,6 +743,62 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Eagle Mountain Roofing | Fort Worth Roofing Contractor</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>eaglemountainroof.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://eaglemountainroof.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>info@eaglemountainroof.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(817) 456-7458</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>86</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>roof repair company Fort Worth TX</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 05:29 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -764,7 +764,6 @@
           <t>https://eaglemountainroof.com/</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>info@eaglemountainroof.com</t>
@@ -794,6 +793,118 @@
         </is>
       </c>
       <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Drain Cleaning | Plumbing Cleaning | Bethlehem, PA</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>buddyplumbs.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://www.buddyplumbs.com/services/drain-cleaning</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>buddyplumbs@gmail.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(484) 379-7028</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>drain cleaning service Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Joliet Plumbing and Sewer Experts</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>jolietplumbingandsewerexperts.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://jolietplumbingandsewerexperts.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>info@indiantypefoundry.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(779)-435-5564</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Joliet IL</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>98</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>sewer repair Joliet IL</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-05 05:32 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -819,7 +819,6 @@
           <t>https://www.buddyplumbs.com/services/drain-cleaning</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>buddyplumbs@gmail.com</t>
@@ -875,7 +874,6 @@
           <t>https://jolietplumbingandsewerexperts.com/</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>info@indiantypefoundry.com</t>
@@ -905,6 +903,66 @@
         </is>
       </c>
       <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Emergency Plumber in Kansas City | The Gentleman Plumber</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>thegentlemanplumberkc.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://www.thegentlemanplumberkc.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Do Moves</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>contactus@tkplumbingkc.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(913) 250-9935</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Kansas City KS</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>emergency plumber Kansas City KS</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-05 05:35 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -968,6 +968,66 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Roofing Services in Brockton, MA | Lema Construction</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>lemaconstructioninc.net</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://lemaconstructioninc.net/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Hardie Alliance</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>info@lemaconstructioninc.net</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(508) 232-1194</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Brockton MA</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>90</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>roofing contractor Brockton MA</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 05:38 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1028,6 +1028,66 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Cool Air California</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>coolaircalifornia.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://coolaircalifornia.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Cool Air</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>coolaircalifornia@gmail.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>424-252-8587</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>AC installation Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 05:49 UTC (cycle 19)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1088,6 +1088,58 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Oftedal Plumbing, LLC | Local Plumber | Billings, MT|</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>oftedalplumbing.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://www.oftedalplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>oftedalplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Billings MT</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>66</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>plumbing company Billings MT</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 05:55 UTC (cycle 23)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1109,13 +1109,11 @@
           <t>https://www.oftedalplumbing.com/</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>oftedalplumbing@gmail.com</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>Billings MT</t>
@@ -1135,6 +1133,66 @@
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BJ Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>bjheatcool.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://bjheatcool.com/louisville-ky-hvac-company/ac-installation/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Air Conditioning</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>office@bjheatcool.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>812-283-7221</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Louisville KY</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>AC installation Louisville KY</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-05 05:58 UTC (cycle 25)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1198,6 +1198,66 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Modestoplumbingpros</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>modestoplumbingpros.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.modestoplumbingpros.com/water-heater-repair-modesto-ca</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Modesto Plumbing</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>example@mysite.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>510-867-0095</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Modesto CA</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>100</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>water heater repair Modesto CA</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 06:04 UTC (cycle 29)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1258,6 +1258,126 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Justin the Plumber</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>justintheplumber.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.justintheplumber.com/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Justin Cannady</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>kyle@justintheplumber.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(904) 524-8188</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>plumber Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Jacksonville Plumbing</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>plumbingjacksonville.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://plumbingjacksonville.com/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Reash Plumbing</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>rollandplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>904.260.7059</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>90</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>plumber Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 06:11 UTC (cycle 34)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1378,6 +1378,174 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Steve Punsky Plumbing</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>stevepunskyplumbing.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://stevepunskyplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>stevepunsky@gmail.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>(207) 615-5001</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Portland ME</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>90</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>plumbing company Portland ME</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Richard P. Waltz Plumbing &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>richardpwaltz.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://richardpwaltz.com/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>info@richardpwaltz.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>(207) 772-2801</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Portland ME</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>86</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>plumbing company Portland ME</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Portland Maine Plumbing &amp; Heating :: Sheldon's Plumbing &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>sheldonsplumbingandheating.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://sheldonsplumbingandheating.com/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>info@sheldonsplumbingandheating.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(207) 799-6211</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Portland ME</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>74</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>plumbing company Portland ME</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 06:17 UTC (cycle 38)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1399,7 +1399,6 @@
           <t>https://stevepunskyplumbing.com/</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>stevepunsky@gmail.com</t>
@@ -1455,7 +1454,6 @@
           <t>https://richardpwaltz.com/</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>info@richardpwaltz.com</t>
@@ -1511,7 +1509,6 @@
           <t>https://sheldonsplumbingandheating.com/</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>info@sheldonsplumbingandheating.com</t>
@@ -1541,6 +1538,62 @@
         </is>
       </c>
       <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Bama Drain and Sewer</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>bamadrainandsewerllc.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://www.bamadrainandsewerllc.com/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>info@bamadrainandsewerllc.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(205) 765-4123</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Tuscaloosa AL</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>72</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>sewer repair Tuscaloosa AL</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-05 06:32 UTC (cycle 48)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1564,7 +1564,6 @@
           <t>https://www.bamadrainandsewerllc.com/</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>info@bamadrainandsewerllc.com</t>
@@ -1594,6 +1593,62 @@
         </is>
       </c>
       <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Philly Roof Find</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>phillyrooffind.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://phillyrooffind.com/philadelphia-pa/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Roofing Contractor</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>admin@phillyrooffind.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Philadelphia PA</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>84</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>roof replacement Philadelphia PA</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-05 06:41 UTC (cycle 54)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1629,7 +1629,6 @@
           <t>admin@phillyrooffind.com</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>Philadelphia PA</t>
@@ -1649,6 +1648,66 @@
         </is>
       </c>
       <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Drain Cleaning Las Vegas | Same-Day | MG Plumbing Services LLC</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>mgplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://mgplumbingservices.com/drain-cleaning-las-vegas/</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Las Vegas</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>admin@mgplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>(702) 480-8070</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>90</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>drain cleaning service Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-05 06:45 UTC (cycle 57)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1713,6 +1713,62 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CTX Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ctxheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.ctxheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>ctxheatingandcooling@gmail.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>254-534-0822</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Round Rock TX</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>86</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>HVAC contractor Round Rock TX</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 06:47 UTC (cycle 58)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1734,7 +1734,6 @@
           <t>https://www.ctxheatingandcooling.com/</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>ctxheatingandcooling@gmail.com</t>
@@ -1764,6 +1763,66 @@
         </is>
       </c>
       <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ranlock Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ranlock.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://www.ranlock.com/roof-replacement/pasadena</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Book Now</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>support@ranlock.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>(281) 299-1086</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>90</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>roof replacement Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-05 06:48 UTC (cycle 59)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1828,6 +1828,62 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Residential Roofing company Long Beach (562) 842-2374</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>longbeachroofing.us</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.longbeachroofing.us/residential-roofing-long-beach-ca</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>info@longbeachroofing.us</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(562) 842-2374</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Long Beach CA</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>98</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>residential roofing company Long Beach CA</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 06:51 UTC (cycle 61)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1849,7 +1849,6 @@
           <t>https://www.longbeachroofing.us/residential-roofing-long-beach-ca</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>info@longbeachroofing.us</t>
@@ -1879,6 +1878,62 @@
         </is>
       </c>
       <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Gartman Mechanical Services</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>gartmanmechanical.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.gartmanmechanical.com/</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>pwilz@gartmanmechanical.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>920-231-5530</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Oshkosh WI</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>64</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>HVAC contractor Oshkosh WI</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-05 06:58 UTC (cycle 66)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1904,7 +1904,6 @@
           <t>https://www.gartmanmechanical.com/</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>pwilz@gartmanmechanical.com</t>
@@ -1934,6 +1933,66 @@
         </is>
       </c>
       <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Atlantic Air Solution</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>atlanticairsolutionsinc.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://atlanticairsolutionsinc.com/coral-springs-ac-installation/</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Atlantic Air</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>atlanticair68@gmail.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>888-886-0969</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>100</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>AC installation Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-05 07:01 UTC (cycle 68)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1998,6 +1998,62 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Quality Plumber | Cedar Rapids, IA | Johnson Plumbing Service</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>johnsonplumbingsvc.com</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://www.johnsonplumbingsvc.com/</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>johnsonplumbing1606@gmail.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>(319) 389-0726</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>86</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>plumber Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 07:10 UTC (cycle 74)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2019,7 +2019,6 @@
           <t>https://www.johnsonplumbingsvc.com/</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>johnsonplumbing1606@gmail.com</t>
@@ -2049,6 +2048,66 @@
         </is>
       </c>
       <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Roofing Services in St. Charles, MO | Brandon J Roofing</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>brandonjroofing.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.brandonjroofing.com/locations/st-charles-mo/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Verified Trusted</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>info@brandonjroofing.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>(636) 288-1040</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>St Charles MO</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>100</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>roofer St Charles MO</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-05 17:01 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L29"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2113,6 +2113,66 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>HVAC in Port St. Lucie, FL</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>portstlucieflhvac.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://portstlucieflhvac.com/</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Port St</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>bloomingdaleproductions@gmail.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>(772) 279-4828</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>92</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>HVAC contractor Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 17:03 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2173,6 +2173,66 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Best HVAC Company in Sandy, UT - Trusted Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>sandyhvacpros.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://sandyhvacpros.com/</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>State St</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>info@sandyhvacpros.com</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>(385) 438-3153</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Sandy UT</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>100</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>heating and cooling company Sandy UT</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 17:11 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2233,6 +2233,62 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Tiger Air Online</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>tigeraironline.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://tigeraironline.com/service-area/furnace-air-conditioning-parma/</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>tigeraironline@gmail.com</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>(440) 598-5050</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Parma OH</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>100</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>air conditioning repair Parma OH</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 17:25 UTC (cycle 18)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2254,7 +2254,6 @@
           <t>https://tigeraironline.com/service-area/furnace-air-conditioning-parma/</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>tigeraironline@gmail.com</t>
@@ -2284,6 +2283,66 @@
         </is>
       </c>
       <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Sure Roofing &amp; Waterproofing, Inc.</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>sureroofing.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://www.sureroofing.com/</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Sure Roofing</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>info@sureroofing.com</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>415-691-1127</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>San Francisco CA</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>88</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>roofer San Francisco CA</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-05 17:30 UTC (cycle 22)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2348,6 +2348,242 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Roofing Company in Olathe, KS | Olathe Roof Pros</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>olatheroofpros.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://olatheroofpros.com/</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>What Olathe</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>hello@olatheroofpros.com</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>(913) 395-4702</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Olathe KS</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>90</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>roofing contractor Olathe KS</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>MR A/C OF ORLANDO</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>mracoforlando.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://mracoforlando.com/</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Central Florida</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>info@mracoforlando.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>321-444-5514</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Orlando FL</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>90</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>AC installation Orlando FL</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Larry Vaught Roofing</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>vaughtroofing.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.vaughtroofing.com/roof-repair/regional-coverage/olathe-roofing-contractor/</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Closed Sunday</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>office@vaughtroofing.com</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>(816) 761-9859</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Olathe KS</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>88</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>roofing contractor Olathe KS</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Hixon Brothers Contracting | Roofing Contractor | Olathe, KS</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>hixonbros.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://www.hixonbros.com/</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>hbc@hixonbros.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>913-782-8499</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Olathe KS</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>82</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>roofing contractor Olathe KS</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 18:07 UTC (cycle 47)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2549,7 +2549,6 @@
           <t>https://www.hixonbros.com/</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>hbc@hixonbros.com</t>
@@ -2579,6 +2578,126 @@
         </is>
       </c>
       <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heat Pump Installation &amp; Repair | Elyria &amp; Lorain County, OH | Anderson Heating </t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>goandersonhvac.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.goandersonhvac.com/heat-pumps/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Common Reasons</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>service@goandersonhvac.com</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>(440) 221-7978</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Lorain OH</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>100</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>heat pump installation Lorain OH</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Downtown Roofing • Cheyenne</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>downtownroofing.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://www.downtownroofing.com/locations/cheyenne</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>At Downtown</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>info@downtownroofing.com</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>(307) 343-0692</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>90</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>roofer Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-05 18:12 UTC (cycle 50)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2703,6 +2703,62 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Sewer line replacement/repair Virginia Beach, VA</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>andersonsplumbingllcva.com</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://andersonsplumbingllcva.com/sewer-line-replacementrepair-virginia-beach-va--andersons-plumbing-6209</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>andersonsplumbing2.0@gmail.com</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>(757) 500-3936</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Virginia Beach VA</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>90</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>sewer repair Virginia Beach VA</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 18:18 UTC (cycle 54)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2724,7 +2724,6 @@
           <t>https://andersonsplumbingllcva.com/sewer-line-replacementrepair-virginia-beach-va--andersons-plumbing-6209</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>andersonsplumbing2.0@gmail.com</t>
@@ -2754,6 +2753,66 @@
         </is>
       </c>
       <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Fox Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>foxhvacpro.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://www.foxhvacpro.com/</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Heating And</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>info@foxhvacpro.com</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>208-398-3188</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Boise ID</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>90</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>heating and cooling company Boise ID</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-05 18:26 UTC (cycle 60)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2818,6 +2818,62 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>service.conditionedairsolutions.com</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>service.conditionedairsolutions.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://service.conditionedairsolutions.com/lp/hvac/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>info@conditionedairsolutions.com</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>(256) 428-1983</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Huntsville AL</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>72</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>furnace repair Huntsville AL</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 18:28 UTC (cycle 61)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2839,7 +2839,6 @@
           <t>https://service.conditionedairsolutions.com/lp/hvac/furnace-repair/</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>info@conditionedairsolutions.com</t>
@@ -2869,6 +2868,66 @@
         </is>
       </c>
       <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Excavate Alaska</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>excavatealaska.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://excavatealaska.com/water-sewer-line-repair/</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Excavate Alaska</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>behappyhomes.officemanager@gmail.com</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>(907) 336-7434</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Anchorage AK</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>90</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>sewer repair Anchorage AK</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-05 19:55 UTC (cycle 120)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2933,6 +2933,62 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Emergency Plumber Jersey City, Newark &amp; Clifton NJ</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>unitedplumbingnj.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://unitedplumbingnj.com/</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>unitedjersey@gmail.com</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>201-222-1555</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Jersey City NJ</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>90</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>emergency plumber Jersey City NJ</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-05 19:59 UTC (cycle 123)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-05.xlsx
+++ b/output/leads_2026-10-05.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2954,7 +2954,6 @@
           <t>https://unitedplumbingnj.com/</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>unitedjersey@gmail.com</t>
@@ -2984,6 +2983,66 @@
         </is>
       </c>
       <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Pacific Coast Elite Plumbing</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>pceplumbing.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://www.pceplumbing.com/areas-we-serve/santa-ana-ca/</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Santa Ana</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>contact@jtsplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>(951) 501-9333</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Santa Ana CA</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>100</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>plumbing company Santa Ana CA</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>

</xml_diff>